<commit_message>
Feature bulk  splicing upload
</commit_message>
<xml_diff>
--- a/Source/SmartInventory/SmartInventory/Content/Templates/Bulk/SplicingConnectionTemplateData.xlsx
+++ b/Source/SmartInventory/SmartInventory/Content/Templates/Bulk/SplicingConnectionTemplateData.xlsx
@@ -4,18 +4,31 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24300" windowHeight="13020" activeTab="1"/>
+    <workbookView windowWidth="19635" windowHeight="7620" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Connections Details" sheetId="1" r:id="rId1"/>
     <sheet name="Guideline - Building Detail" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="39">
   <si>
     <t>source_network_id</t>
   </si>
@@ -41,6 +54,12 @@
     <t>destination_port_type</t>
   </si>
   <si>
+    <t>connector_id</t>
+  </si>
+  <si>
+    <t>connector_type</t>
+  </si>
+  <si>
     <t>Very IMP: Do not Delete/Update any column header in Building_Detail Sheet</t>
   </si>
   <si>
@@ -105,6 +124,18 @@
   </si>
   <si>
     <t>destination port type</t>
+  </si>
+  <si>
+    <t>Connector_id</t>
+  </si>
+  <si>
+    <t>Connector_network_id.</t>
+  </si>
+  <si>
+    <t>Connector_type</t>
+  </si>
+  <si>
+    <t>Connector type</t>
   </si>
   <si>
     <t>Port Type</t>
@@ -119,12 +150,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -165,10 +196,50 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -180,6 +251,53 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -187,129 +305,42 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -336,13 +367,145 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -354,61 +517,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -420,103 +541,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -545,11 +570,65 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -578,36 +657,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -618,181 +667,157 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -806,58 +831,61 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="40% - Accent1" xfId="1" builtinId="31"/>
-    <cellStyle name="Comma" xfId="2" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="3" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
-    <cellStyle name="Currency" xfId="5" builtinId="4"/>
-    <cellStyle name="Percent" xfId="6" builtinId="5"/>
-    <cellStyle name="Check Cell" xfId="7" builtinId="23"/>
-    <cellStyle name="Heading 2" xfId="8" builtinId="17"/>
-    <cellStyle name="Note" xfId="9" builtinId="10"/>
-    <cellStyle name="Hyperlink" xfId="10" builtinId="8"/>
-    <cellStyle name="60% - Accent4" xfId="11" builtinId="44"/>
-    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9"/>
-    <cellStyle name="40% - Accent3" xfId="13" builtinId="39"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11"/>
-    <cellStyle name="40% - Accent2" xfId="15" builtinId="35"/>
-    <cellStyle name="Title" xfId="16" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="17" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="18" builtinId="16"/>
-    <cellStyle name="Heading 3" xfId="19" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="20" builtinId="19"/>
-    <cellStyle name="Input" xfId="21" builtinId="20"/>
-    <cellStyle name="60% - Accent3" xfId="22" builtinId="40"/>
-    <cellStyle name="Good" xfId="23" builtinId="26"/>
-    <cellStyle name="Output" xfId="24" builtinId="21"/>
-    <cellStyle name="20% - Accent1" xfId="25" builtinId="30"/>
-    <cellStyle name="Calculation" xfId="26" builtinId="22"/>
-    <cellStyle name="Linked Cell" xfId="27" builtinId="24"/>
-    <cellStyle name="Total" xfId="28" builtinId="25"/>
-    <cellStyle name="Bad" xfId="29" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="30" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="31" builtinId="29"/>
-    <cellStyle name="20% - Accent5" xfId="32" builtinId="46"/>
-    <cellStyle name="60% - Accent1" xfId="33" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="34" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="35" builtinId="34"/>
-    <cellStyle name="20% - Accent6" xfId="36" builtinId="50"/>
-    <cellStyle name="60% - Accent2" xfId="37" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="38" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="39" builtinId="38"/>
-    <cellStyle name="Accent4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="42" builtinId="43"/>
-    <cellStyle name="Accent5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - Accent5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="45" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="46" builtinId="49"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
@@ -1128,8 +1156,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="7"/>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.5714285714286" customWidth="1"/>
     <col min="2" max="2" width="19.8571428571429" customWidth="1"/>
@@ -1139,9 +1167,10 @@
     <col min="6" max="6" width="24.5714285714286" customWidth="1"/>
     <col min="7" max="7" width="20.8571428571429" customWidth="1"/>
     <col min="8" max="8" width="24.1428571428571" customWidth="1"/>
+    <col min="9" max="9" width="16.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1165,6 +1194,12 @@
       </c>
       <c r="H1" t="s">
         <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1176,7 +1211,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="E6:I21"/>
+  <dimension ref="E6:I22"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <cols>
     <col min="5" max="5" width="48.8571428571429" customWidth="1"/>
@@ -1188,7 +1223,7 @@
   <sheetData>
     <row r="6" spans="5:9">
       <c r="E6" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -1197,7 +1232,7 @@
     </row>
     <row r="7" ht="21" spans="5:9">
       <c r="E7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1206,19 +1241,19 @@
     </row>
     <row r="8" spans="5:9">
       <c r="E8" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" ht="43" customHeight="1" spans="5:9">
@@ -1226,16 +1261,16 @@
         <v>0</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="5:9">
@@ -1243,16 +1278,16 @@
         <v>1</v>
       </c>
       <c r="F10" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="I10" s="4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="5:9">
@@ -1260,13 +1295,13 @@
         <v>2</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I11" s="4">
         <v>12</v>
@@ -1277,16 +1312,16 @@
         <v>3</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" ht="30" spans="5:9">
@@ -1294,16 +1329,16 @@
         <v>4</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="5:9">
@@ -1311,16 +1346,16 @@
         <v>5</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="5:9">
@@ -1328,13 +1363,13 @@
         <v>6</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I15" s="4">
         <v>12</v>
@@ -1345,38 +1380,57 @@
         <v>7</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="5:9">
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
     </row>
-    <row r="19" spans="5:5">
-      <c r="E19" s="5" t="s">
-        <v>30</v>
-      </c>
+    <row r="18" spans="5:9">
+      <c r="E18" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
     </row>
     <row r="20" spans="5:5">
-      <c r="E20" s="5" t="s">
-        <v>31</v>
+      <c r="E20" s="6" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="5:5">
-      <c r="E21" s="5" t="s">
-        <v>32</v>
+      <c r="E21" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="5:5">
+      <c r="E22" s="6" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>